<commit_message>
auxcorrection, gebeurd/beuren -> gebeurd/gebeuren
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/ASTA_Index_Current.xlsx
+++ b/src/sastadev/data/methods/ASTA_Index_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D7372D5-D43A-4FEF-A4CC-18F6AD3C5CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1607D955-18F4-4276-8BB4-149D4C1344AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="209">
   <si>
     <t>ID</t>
   </si>
@@ -635,9 +635,6 @@
     <t>//node[@pt="ww" and %ASTA_modalww% and not(%ASTA_XXX%)]</t>
   </si>
   <si>
-    <t>get_missing_det</t>
-  </si>
-  <si>
     <t xml:space="preserve"> deletie van een lidwoord;tijdelijk uitgezet</t>
   </si>
   <si>
@@ -651,6 +648,21 @@
   </si>
   <si>
     <t>implied_by</t>
+  </si>
+  <si>
+    <t>asta_dellid</t>
+  </si>
+  <si>
+    <t>sublid</t>
+  </si>
+  <si>
+    <t>congruentiefout</t>
+  </si>
+  <si>
+    <t>A052</t>
+  </si>
+  <si>
+    <t>pv_regionale_vorm</t>
   </si>
 </sst>
 </file>
@@ -1065,10 +1077,10 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>202</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>8</v>
@@ -1098,10 +1110,10 @@
         <v>182</v>
       </c>
       <c r="T1" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>203</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>204</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>183</v>
@@ -1332,6 +1344,9 @@
       <c r="O9" t="s">
         <v>128</v>
       </c>
+      <c r="R9" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -1482,11 +1497,17 @@
       <c r="H15" t="s">
         <v>14</v>
       </c>
+      <c r="L15" t="s">
+        <v>206</v>
+      </c>
       <c r="M15" t="s">
         <v>14</v>
       </c>
       <c r="O15" t="s">
         <v>128</v>
+      </c>
+      <c r="W15" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.3">
@@ -1763,6 +1784,9 @@
       <c r="O25" t="s">
         <v>128</v>
       </c>
+      <c r="R25" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
@@ -1921,6 +1945,9 @@
       <c r="H32" t="s">
         <v>14</v>
       </c>
+      <c r="L32" t="s">
+        <v>205</v>
+      </c>
       <c r="M32" t="s">
         <v>14</v>
       </c>
@@ -1947,6 +1974,9 @@
       <c r="H33" t="s">
         <v>14</v>
       </c>
+      <c r="L33" t="s">
+        <v>204</v>
+      </c>
       <c r="M33" t="s">
         <v>14</v>
       </c>
@@ -1954,10 +1984,10 @@
         <v>128</v>
       </c>
       <c r="W33" t="s">
+        <v>204</v>
+      </c>
+      <c r="X33" t="s">
         <v>199</v>
-      </c>
-      <c r="X33" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="34" spans="1:24" x14ac:dyDescent="0.3">
@@ -2365,7 +2395,30 @@
       </c>
     </row>
     <row r="50" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="E50" s="4"/>
+      <c r="A50" t="s">
+        <v>207</v>
+      </c>
+      <c r="D50" t="s">
+        <v>192</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="H50" t="s">
+        <v>118</v>
+      </c>
+      <c r="L50" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="M50" t="s">
+        <v>14</v>
+      </c>
+      <c r="O50" t="s">
+        <v>128</v>
+      </c>
+      <c r="X50" s="4" t="s">
+        <v>208</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:Z49" xr:uid="{356449EB-3FBE-4443-8528-03CDC854A576}"/>

</xml_diff>

<commit_message>
Reporting of several grammatical errors, esp. in STAP
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/ASTA_Index_Current.xlsx
+++ b/src/sastadev/data/methods/ASTA_Index_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1607D955-18F4-4276-8BB4-149D4C1344AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A34CB864-5580-4F49-87F5-9BF82E38C386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="212">
   <si>
     <t>ID</t>
   </si>
@@ -663,6 +663,15 @@
   </si>
   <si>
     <t>pv_regionale_vorm</t>
+  </si>
+  <si>
+    <t>A053</t>
+  </si>
+  <si>
+    <t>adj_agr_fout</t>
+  </si>
+  <si>
+    <t>adj_agreement_errors</t>
   </si>
 </sst>
 </file>
@@ -1042,7 +1051,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z50"/>
+  <dimension ref="A1:Z51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
@@ -2420,6 +2429,32 @@
         <v>208</v>
       </c>
     </row>
+    <row r="51" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>209</v>
+      </c>
+      <c r="D51" t="s">
+        <v>192</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="H51" t="s">
+        <v>118</v>
+      </c>
+      <c r="L51" t="s">
+        <v>211</v>
+      </c>
+      <c r="M51" t="s">
+        <v>14</v>
+      </c>
+      <c r="O51" t="s">
+        <v>128</v>
+      </c>
+      <c r="X51" t="s">
+        <v>211</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Z49" xr:uid="{356449EB-3FBE-4443-8528-03CDC854A576}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O28">

</xml_diff>